<commit_message>
fix: place regenerated artifacts in correct gtm/ folders (new $1,500 pricing)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gtm/03-pricing-billing/Verispect-Financial-Model.xlsx
+++ b/gtm/03-pricing-billing/Verispect-Financial-Model.xlsx
@@ -554,11 +554,11 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>99</v>
+        <v>1500</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>self-serve workhorse</t>
+          <t>Verispect standard, $/mo</t>
         </is>
       </c>
     </row>
@@ -569,11 +569,11 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>399</v>
+        <v>1500</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>scale-up / enterprise-facing</t>
+          <t>Founding rate locked (rises to 2500)</t>
         </is>
       </c>
     </row>
@@ -584,11 +584,11 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>custom 2k-10k, avg modeled</t>
+          <t>multi-entity/SSO/SLA, avg modeled</t>
         </is>
       </c>
     </row>
@@ -2289,17 +2289,17 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Price / mo (€)</t>
+          <t>Price / mo ($)</t>
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>99</v>
+        <v>1500</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>399</v>
+        <v>1500</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="6">

</xml_diff>